<commit_message>
ZIP codes kept in their province range, Philippine address on the migration workbook clients, address component test, API export and templates rebuilt
</commit_message>
<xml_diff>
--- a/docs/package/05_Delivery/Upload_Templates/GoLive_Migration_Workbook.xlsx
+++ b/docs/package/05_Delivery/Upload_Templates/GoLive_Migration_Workbook.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="309">
   <si>
     <t xml:space="preserve">Item</t>
   </si>
@@ -316,22 +316,34 @@
     <t xml:space="preserve">Clients: Address</t>
   </si>
   <si>
-    <t xml:space="preserve">Optional. Street address</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clients: City</t>
+    <t xml:space="preserve">Optional. House / unit no. and street</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clients: Barangay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clients: City / Municipality</t>
   </si>
   <si>
     <t xml:space="preserve">Clients: Province</t>
   </si>
   <si>
+    <t xml:space="preserve">Optional. Province of the Province master (Metro Manila for NCR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clients: Region</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. Filled from the province when empty</t>
+  </si>
+  <si>
     <t xml:space="preserve">Clients: Country</t>
   </si>
   <si>
     <t xml:space="preserve">Optional. Philippines when empty</t>
   </si>
   <si>
-    <t xml:space="preserve">Clients: Postal Code</t>
+    <t xml:space="preserve">Clients: ZIP Code</t>
   </si>
   <si>
     <t xml:space="preserve">Policies: Policy Number</t>
@@ -715,16 +727,22 @@
     <t xml:space="preserve">Address</t>
   </si>
   <si>
-    <t xml:space="preserve">City</t>
+    <t xml:space="preserve">Barangay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">City / Municipality</t>
   </si>
   <si>
     <t xml:space="preserve">Province</t>
   </si>
   <si>
+    <t xml:space="preserve">Region</t>
+  </si>
+  <si>
     <t xml:space="preserve">Country</t>
   </si>
   <si>
-    <t xml:space="preserve">Postal Code</t>
+    <t xml:space="preserve">ZIP Code</t>
   </si>
   <si>
     <t xml:space="preserve">SAMPLE C-000123</t>
@@ -748,13 +766,19 @@
     <t xml:space="preserve">1988-04-12</t>
   </si>
   <si>
-    <t xml:space="preserve">12 Mabini St., San Antonio</t>
+    <t xml:space="preserve">Unit 4B, 12 Mabini St.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">San Antonio</t>
   </si>
   <si>
     <t xml:space="preserve">Pasig City</t>
   </si>
   <si>
     <t xml:space="preserve">Metro Manila</t>
+  </si>
+  <si>
+    <t xml:space="preserve">National Capital Region (NCR)</t>
   </si>
   <si>
     <t xml:space="preserve">Philippines</t>
@@ -1048,7 +1072,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B95"/>
+  <dimension ref="A1:B97"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -1516,23 +1540,23 @@
         <v>104</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="0" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="0" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>108</v>
+        <v>91</v>
       </c>
     </row>
     <row r="63">
@@ -1708,23 +1732,23 @@
         <v>151</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>120</v>
+        <v>152</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="0" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="0" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>155</v>
+        <v>124</v>
       </c>
     </row>
     <row r="87">
@@ -1740,20 +1764,20 @@
         <v>158</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>91</v>
+        <v>159</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="0" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="0" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B90" s="4" t="s">
         <v>91</v>
@@ -1761,18 +1785,18 @@
     </row>
     <row r="91">
       <c r="A91" s="0" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="0" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>165</v>
+        <v>91</v>
       </c>
     </row>
     <row r="93">
@@ -1797,6 +1821,22 @@
       </c>
       <c r="B95" s="4" t="s">
         <v>171</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="0" t="s">
+        <v>172</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="0" t="s">
+        <v>174</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>175</v>
       </c>
     </row>
   </sheetData>
@@ -1819,104 +1859,104 @@
   <sheetData>
     <row r="1" spans="1:6" ht="20" customHeight="1">
       <c r="A1" s="8" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="11" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="11"/>
       <c r="B4" s="11"/>
       <c r="C4" s="11" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="D4" s="11"/>
       <c r="E4" s="11" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="11"/>
       <c r="B5" s="11"/>
       <c r="C5" s="11" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="D5" s="11"/>
       <c r="E5" s="11" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11"/>
       <c r="B6" s="11"/>
       <c r="C6" s="11" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="D6" s="11"/>
       <c r="E6" s="11" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="7">
@@ -1925,10 +1965,10 @@
       <c r="C7" s="11"/>
       <c r="D7" s="11"/>
       <c r="E7" s="11" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
     </row>
     <row r="8">
@@ -1937,10 +1977,10 @@
       <c r="C8" s="11"/>
       <c r="D8" s="11"/>
       <c r="E8" s="11" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
     </row>
     <row r="9">
@@ -1949,10 +1989,10 @@
       <c r="C9" s="11"/>
       <c r="D9" s="11"/>
       <c r="E9" s="11" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
     </row>
     <row r="10">
@@ -1961,10 +2001,10 @@
       <c r="C10" s="11"/>
       <c r="D10" s="11"/>
       <c r="E10" s="11" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
     </row>
     <row r="11">
@@ -1973,10 +2013,10 @@
       <c r="C11" s="11"/>
       <c r="D11" s="11"/>
       <c r="E11" s="11" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
     </row>
     <row r="12">
@@ -1985,10 +2025,10 @@
       <c r="C12" s="11"/>
       <c r="D12" s="11"/>
       <c r="E12" s="11" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="13">
@@ -1997,10 +2037,10 @@
       <c r="C13" s="11"/>
       <c r="D13" s="11"/>
       <c r="E13" s="11" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
     </row>
     <row r="14">
@@ -2009,10 +2049,10 @@
       <c r="C14" s="11"/>
       <c r="D14" s="11"/>
       <c r="E14" s="11" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
     </row>
     <row r="15">
@@ -2022,7 +2062,7 @@
       <c r="D15" s="11"/>
       <c r="E15" s="11"/>
       <c r="F15" s="11" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
     </row>
     <row r="16">
@@ -2032,7 +2072,7 @@
       <c r="D16" s="11"/>
       <c r="E16" s="11"/>
       <c r="F16" s="11" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="17">
@@ -2042,7 +2082,7 @@
       <c r="D17" s="11"/>
       <c r="E17" s="11"/>
       <c r="F17" s="11" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
     </row>
     <row r="18">
@@ -2052,7 +2092,7 @@
       <c r="D18" s="11"/>
       <c r="E18" s="11"/>
       <c r="F18" s="11" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
     </row>
     <row r="19">
@@ -2062,7 +2102,7 @@
       <c r="D19" s="11"/>
       <c r="E19" s="11"/>
       <c r="F19" s="11" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
     </row>
     <row r="20">
@@ -2072,7 +2112,7 @@
       <c r="D20" s="11"/>
       <c r="E20" s="11"/>
       <c r="F20" s="11" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
     </row>
   </sheetData>
@@ -2082,7 +2122,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="17" style="11" customWidth="1"/>
@@ -2097,99 +2137,113 @@
     <col min="10" max="10" width="14" style="11" customWidth="1"/>
     <col min="11" max="11" width="14" style="11" customWidth="1"/>
     <col min="12" max="12" width="14" style="11" customWidth="1"/>
-    <col min="13" max="13" width="14" style="11" customWidth="1"/>
+    <col min="13" max="13" width="25" style="11" customWidth="1"/>
     <col min="14" max="14" width="14" style="11" customWidth="1"/>
-    <col min="15" max="15" width="17" style="11" customWidth="1"/>
+    <col min="15" max="15" width="14" style="11" customWidth="1"/>
+    <col min="16" max="16" width="14" style="11" customWidth="1"/>
+    <col min="17" max="17" width="14" style="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="20" customHeight="1">
+    <row r="1" spans="1:17" ht="20" customHeight="1">
       <c r="A1" s="8" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="L1" s="8" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="M1" s="8" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="N1" s="8" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="O1" s="8" t="s">
-        <v>235</v>
+        <v>239</v>
+      </c>
+      <c r="P1" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="Q1" s="8" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="E2" s="9"/>
       <c r="F2" s="9" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="J2" s="9"/>
       <c r="K2" s="9" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="L2" s="9" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="M2" s="9" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="N2" s="9" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="O2" s="9" t="s">
-        <v>247</v>
+        <v>253</v>
+      </c>
+      <c r="P2" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="Q2" s="9" t="s">
+        <v>255</v>
       </c>
     </row>
   </sheetData>
@@ -2227,95 +2281,95 @@
   <sheetData>
     <row r="1" spans="1:16" ht="20" customHeight="1">
       <c r="A1" s="8" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="L1" s="8" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="M1" s="8" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="N1" s="8" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="O1" s="8" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="P1" s="8" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E2" s="9"/>
       <c r="F2" s="9" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="J2" s="9" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="K2" s="9" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="L2" s="9"/>
       <c r="M2" s="9" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="N2" s="9" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="O2" s="9" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
       <c r="P2" s="9"/>
     </row>
@@ -2352,36 +2406,36 @@
   <sheetData>
     <row r="1" spans="1:5" ht="20" customHeight="1">
       <c r="A1" s="8" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
     </row>
   </sheetData>
@@ -2408,63 +2462,63 @@
   <sheetData>
     <row r="1" spans="1:10" ht="20" customHeight="1">
       <c r="A1" s="8" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>280</v>
+        <v>288</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="J1" s="8" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="J2" s="9"/>
     </row>
@@ -2491,27 +2545,27 @@
   <sheetData>
     <row r="1" spans="1:4" ht="20" customHeight="1">
       <c r="A1" s="8" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>296</v>
+        <v>304</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>299</v>
+        <v>307</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>300</v>
+        <v>308</v>
       </c>
       <c r="D2" s="9"/>
     </row>

</xml_diff>

<commit_message>
Document the layout screens and the withdrawn screens
User manual 1.2.5: E-mail Layout, Documents and Reports Layout and
Document Signatures replace Theme and Branding, System Settings keeps
the display currency and the language, the Data Privacy section and
panels go (the masking of personal identifiers stays) and the Go-Live
Data Load chapter describes the workbooks loaded through the API, with
new screenshots; the in-app help is rebuilt. The branding guide, the
brand pack README (zip rebuilt), the deployment guides, the developer
guide and the upload templates follow; the API reference is exported
again and the accounting README says how the cost centre screen reads
its master.
</commit_message>
<xml_diff>
--- a/docs/package/05_Delivery/Upload_Templates/GoLive_Migration_Workbook.xlsx
+++ b/docs/package/05_Delivery/Upload_Templates/GoLive_Migration_Workbook.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="301">
   <si>
     <t xml:space="preserve">Item</t>
   </si>
@@ -34,10 +34,10 @@
     <t xml:space="preserve">Blank template: fill in the object sheets.</t>
   </si>
   <si>
-    <t xml:space="preserve">Upload on</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Master &gt; Go-Live Data Load (System Administrator). API: POST /api/data-load/batches (multipart field "file", field kit).</t>
+    <t xml:space="preserve">Upload with</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API: POST /api/data-load/batches (multipart field "file", field kit), System Administrator; the go-live scripts (npm run rehearsal:golive) use it.</t>
   </si>
   <si>
     <t xml:space="preserve">Cutover date</t>
@@ -580,7 +580,7 @@
     <t xml:space="preserve">APEX</t>
   </si>
   <si>
-    <t xml:space="preserve">BOND</t>
+    <t xml:space="preserve">CL-COMP</t>
   </si>
   <si>
     <t xml:space="preserve">corporate</t>
@@ -595,103 +595,79 @@
     <t xml:space="preserve">in-review</t>
   </si>
   <si>
+    <t xml:space="preserve">AXA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CL-VOL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partial</t>
+  </si>
+  <si>
     <t xml:space="preserve">EVERSAFE</t>
   </si>
   <si>
-    <t xml:space="preserve">BURGLARY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Partial</t>
+    <t xml:space="preserve">CTPL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Completed</t>
   </si>
   <si>
     <t xml:space="preserve">FPG</t>
   </si>
   <si>
-    <t xml:space="preserve">CAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Completed</t>
+    <t xml:space="preserve">GPA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Refunded</t>
   </si>
   <si>
     <t xml:space="preserve">GOLDENHORIZON</t>
   </si>
   <si>
-    <t xml:space="preserve">CGL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Refunded</t>
+    <t xml:space="preserve">MOTOR</t>
   </si>
   <si>
     <t xml:space="preserve">INTEGRITY</t>
   </si>
   <si>
-    <t xml:space="preserve">CTPL</t>
+    <t xml:space="preserve">PA</t>
   </si>
   <si>
     <t xml:space="preserve">LIBERTYSHIELD</t>
   </si>
   <si>
-    <t xml:space="preserve">EAR</t>
+    <t xml:space="preserve">PARCEL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAAGAP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRAVEL</t>
   </si>
   <si>
     <t xml:space="preserve">MALAYAN</t>
   </si>
   <si>
-    <t xml:space="preserve">EB</t>
-  </si>
-  <si>
     <t xml:space="preserve">MAPFRE</t>
   </si>
   <si>
-    <t xml:space="preserve">FIRE</t>
-  </si>
-  <si>
     <t xml:space="preserve">MERCANTILE</t>
   </si>
   <si>
-    <t xml:space="preserve">GPA</t>
-  </si>
-  <si>
     <t xml:space="preserve">PIONEER</t>
   </si>
   <si>
-    <t xml:space="preserve">HOME</t>
-  </si>
-  <si>
     <t xml:space="preserve">SECUREGUARD</t>
   </si>
   <si>
-    <t xml:space="preserve">HULL</t>
-  </si>
-  <si>
     <t xml:space="preserve">SENTINEL</t>
   </si>
   <si>
-    <t xml:space="preserve">IAR</t>
-  </si>
-  <si>
     <t xml:space="preserve">STANDARD</t>
   </si>
   <si>
-    <t xml:space="preserve">MARINE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MICRO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MONEY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MOTOR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TRAVEL</t>
+    <t xml:space="preserve">STRONGHOLD</t>
   </si>
   <si>
     <t xml:space="preserve">Client Code *</t>
@@ -953,7 +929,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -980,8 +956,42 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF0B2A4A"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF5F6B76"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1009,6 +1019,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF4CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1040,9 +1068,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1063,6 +1091,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1846,7 +1881,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15" style="11" customWidth="1"/>
@@ -2003,9 +2038,7 @@
       <c r="E10" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="F10" s="11" t="s">
-        <v>210</v>
-      </c>
+      <c r="F10" s="11"/>
     </row>
     <row r="11">
       <c r="A11" s="11"/>
@@ -2013,11 +2046,9 @@
       <c r="C11" s="11"/>
       <c r="D11" s="11"/>
       <c r="E11" s="11" t="s">
-        <v>211</v>
-      </c>
-      <c r="F11" s="11" t="s">
-        <v>212</v>
-      </c>
+        <v>210</v>
+      </c>
+      <c r="F11" s="11"/>
     </row>
     <row r="12">
       <c r="A12" s="11"/>
@@ -2025,11 +2056,9 @@
       <c r="C12" s="11"/>
       <c r="D12" s="11"/>
       <c r="E12" s="11" t="s">
-        <v>213</v>
-      </c>
-      <c r="F12" s="11" t="s">
-        <v>214</v>
-      </c>
+        <v>211</v>
+      </c>
+      <c r="F12" s="11"/>
     </row>
     <row r="13">
       <c r="A13" s="11"/>
@@ -2037,11 +2066,9 @@
       <c r="C13" s="11"/>
       <c r="D13" s="11"/>
       <c r="E13" s="11" t="s">
-        <v>215</v>
-      </c>
-      <c r="F13" s="11" t="s">
-        <v>216</v>
-      </c>
+        <v>212</v>
+      </c>
+      <c r="F13" s="11"/>
     </row>
     <row r="14">
       <c r="A14" s="11"/>
@@ -2049,71 +2076,39 @@
       <c r="C14" s="11"/>
       <c r="D14" s="11"/>
       <c r="E14" s="11" t="s">
-        <v>217</v>
-      </c>
-      <c r="F14" s="11" t="s">
-        <v>218</v>
-      </c>
+        <v>213</v>
+      </c>
+      <c r="F14" s="11"/>
     </row>
     <row r="15">
       <c r="A15" s="11"/>
       <c r="B15" s="11"/>
       <c r="C15" s="11"/>
       <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11" t="s">
-        <v>219</v>
-      </c>
+      <c r="E15" s="11" t="s">
+        <v>214</v>
+      </c>
+      <c r="F15" s="11"/>
     </row>
     <row r="16">
       <c r="A16" s="11"/>
       <c r="B16" s="11"/>
       <c r="C16" s="11"/>
       <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11" t="s">
-        <v>220</v>
-      </c>
+      <c r="E16" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="F16" s="11"/>
     </row>
     <row r="17">
       <c r="A17" s="11"/>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
       <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="11"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="11"/>
-      <c r="B19" s="11"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="11"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11" t="s">
-        <v>224</v>
-      </c>
+      <c r="E17" s="11" t="s">
+        <v>216</v>
+      </c>
+      <c r="F17" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2146,104 +2141,104 @@
   <sheetData>
     <row r="1" spans="1:17" ht="20" customHeight="1">
       <c r="A1" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="I1" s="8" t="s">
         <v>225</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="J1" s="8" t="s">
         <v>226</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="K1" s="8" t="s">
         <v>227</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="L1" s="8" t="s">
         <v>228</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="M1" s="8" t="s">
         <v>229</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="N1" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="O1" s="8" t="s">
         <v>231</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="P1" s="8" t="s">
         <v>232</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="Q1" s="8" t="s">
         <v>233</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>234</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>235</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>236</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>237</v>
-      </c>
-      <c r="N1" s="8" t="s">
-        <v>238</v>
-      </c>
-      <c r="O1" s="8" t="s">
-        <v>239</v>
-      </c>
-      <c r="P1" s="8" t="s">
-        <v>240</v>
-      </c>
-      <c r="Q1" s="8" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>182</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="E2" s="9"/>
       <c r="F2" s="9" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="J2" s="9"/>
       <c r="K2" s="9" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="L2" s="9" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="M2" s="9" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="N2" s="9" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="O2" s="9" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="P2" s="9" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="Q2" s="9" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
     </row>
   </sheetData>
@@ -2281,40 +2276,40 @@
   <sheetData>
     <row r="1" spans="1:16" ht="20" customHeight="1">
       <c r="A1" s="8" t="s">
+        <v>248</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>217</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>256</v>
       </c>
-      <c r="B1" s="8" t="s">
-        <v>225</v>
-      </c>
-      <c r="C1" s="8" t="s">
+      <c r="K1" s="8" t="s">
         <v>257</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="L1" s="8" t="s">
         <v>258</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>259</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>260</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>261</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>262</v>
-      </c>
-      <c r="I1" s="8" t="s">
-        <v>263</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>264</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>265</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>266</v>
       </c>
       <c r="M1" s="8" t="s">
         <v>177</v>
@@ -2323,43 +2318,43 @@
         <v>178</v>
       </c>
       <c r="O1" s="8" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
       <c r="P1" s="8" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>222</v>
+        <v>202</v>
       </c>
       <c r="E2" s="9"/>
       <c r="F2" s="9" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="J2" s="9" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
       <c r="K2" s="9" t="s">
-        <v>276</v>
+        <v>268</v>
       </c>
       <c r="L2" s="9"/>
       <c r="M2" s="9" t="s">
@@ -2369,17 +2364,17 @@
         <v>197</v>
       </c>
       <c r="O2" s="9" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="P2" s="9"/>
     </row>
   </sheetData>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showErrorMessage="0" errorStyle="information" sqref="C2:C5000">
-      <formula1>Lists!$E$2:$E$14</formula1>
+      <formula1>Lists!$E$2:$E$17</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="0" errorStyle="information" sqref="D2:D5000">
-      <formula1>Lists!$F$2:$F$20</formula1>
+      <formula1>Lists!$F$2:$F$9</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" sqref="M2:M5000">
       <formula1>Lists!$B$2:$B$3</formula1>
@@ -2406,36 +2401,36 @@
   <sheetData>
     <row r="1" spans="1:5" ht="20" customHeight="1">
       <c r="A1" s="8" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>279</v>
+        <v>271</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>283</v>
+        <v>275</v>
       </c>
       <c r="D2" s="9" t="s">
+        <v>268</v>
+      </c>
+      <c r="E2" s="9" t="s">
         <v>276</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>284</v>
       </c>
     </row>
   </sheetData>
@@ -2462,63 +2457,63 @@
   <sheetData>
     <row r="1" spans="1:10" ht="20" customHeight="1">
       <c r="A1" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>248</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>278</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>279</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>283</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>284</v>
+      </c>
+      <c r="J1" s="8" t="s">
         <v>285</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>256</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>286</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>287</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>288</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>289</v>
-      </c>
-      <c r="G1" s="8" t="s">
-        <v>290</v>
-      </c>
-      <c r="H1" s="8" t="s">
-        <v>291</v>
-      </c>
-      <c r="I1" s="8" t="s">
-        <v>292</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>295</v>
+        <v>287</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="E2" s="9" t="s">
         <v>191</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>299</v>
+        <v>291</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>301</v>
+        <v>293</v>
       </c>
       <c r="J2" s="9"/>
     </row>
@@ -2545,27 +2540,27 @@
   <sheetData>
     <row r="1" spans="1:4" ht="20" customHeight="1">
       <c r="A1" s="8" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>303</v>
+        <v>295</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>304</v>
+        <v>296</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>305</v>
+        <v>297</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="s">
-        <v>306</v>
+        <v>298</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>307</v>
+        <v>299</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>308</v>
+        <v>300</v>
       </c>
       <c r="D2" s="9"/>
     </row>

</xml_diff>